<commit_message>
Fix inconsistencies between alias files and lineage definitions.
</commit_message>
<xml_diff>
--- a/tabular/reference/ervr/ervr_alias.xlsx
+++ b/tabular/reference/ervr/ervr_alias.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rob/Projects/erv/locus-level/ERVdb-HomoSapiens/tabular/reference/ervr/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B087C047-CB61-B749-87F6-AF53DE2D67E6}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{694E38F2-7539-564F-BFC7-33B1861EA986}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2960" yWindow="2260" windowWidth="22740" windowHeight="14760" xr2:uid="{E2A31913-0241-5047-ACED-7542084468C7}"/>
+    <workbookView xWindow="2540" yWindow="940" windowWidth="14240" windowHeight="17060" xr2:uid="{E2A31913-0241-5047-ACED-7542084468C7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="61">
   <si>
     <t>erv_lineage.id</t>
   </si>
@@ -71,18 +71,6 @@
     <t>HERV19</t>
   </si>
   <si>
-    <t>HERV-31</t>
-  </si>
-  <si>
-    <t>ERV3-1</t>
-  </si>
-  <si>
-    <t>HERV-35</t>
-  </si>
-  <si>
-    <t>HERV35</t>
-  </si>
-  <si>
     <t>HERV-G25</t>
   </si>
   <si>
@@ -113,12 +101,6 @@
     <t>LOR1</t>
   </si>
   <si>
-    <t>LTR-37</t>
-  </si>
-  <si>
-    <t>LTR37</t>
-  </si>
-  <si>
     <t>LTR-43</t>
   </si>
   <si>
@@ -131,54 +113,6 @@
     <t>MER101</t>
   </si>
   <si>
-    <t>MER-21</t>
-  </si>
-  <si>
-    <t>MER21</t>
-  </si>
-  <si>
-    <t>MER-31</t>
-  </si>
-  <si>
-    <t>MER31</t>
-  </si>
-  <si>
-    <t>MER-34B</t>
-  </si>
-  <si>
-    <t>MER34B</t>
-  </si>
-  <si>
-    <t>MER-41</t>
-  </si>
-  <si>
-    <t>MER41</t>
-  </si>
-  <si>
-    <t>MER-57</t>
-  </si>
-  <si>
-    <t>MER57</t>
-  </si>
-  <si>
-    <t>MER57A</t>
-  </si>
-  <si>
-    <t>MER-61</t>
-  </si>
-  <si>
-    <t>MER61</t>
-  </si>
-  <si>
-    <t>MER-65</t>
-  </si>
-  <si>
-    <t>MER65</t>
-  </si>
-  <si>
-    <t>mer65</t>
-  </si>
-  <si>
     <t>MER-70</t>
   </si>
   <si>
@@ -227,60 +161,9 @@
     <t>ERVR-3.Lambda.16A3</t>
   </si>
   <si>
-    <t>ERV-3.Lambda.16</t>
-  </si>
-  <si>
-    <t>ERV-1.Zeta.19</t>
-  </si>
-  <si>
-    <t>ERV-1.Rho.Rb.31</t>
-  </si>
-  <si>
-    <t>ERV-1.Zeta.35</t>
-  </si>
-  <si>
-    <t>ERV-1.Zeta.W9P.P.G25</t>
-  </si>
-  <si>
-    <t>ERV-3.Lambda.40</t>
-  </si>
-  <si>
-    <t>ERV-3.Lambda.53</t>
-  </si>
-  <si>
-    <t>ERVR-1.Theta.LOR1</t>
-  </si>
-  <si>
-    <t>ERVR-1.Theta.37</t>
-  </si>
-  <si>
     <t>ERVR-1.Theta.43</t>
   </si>
   <si>
-    <t>ERVR-1.Theta.101</t>
-  </si>
-  <si>
-    <t>ERVR-1.Theta.MER21</t>
-  </si>
-  <si>
-    <t>ERVR-1.Theta.MER31</t>
-  </si>
-  <si>
-    <t>ERVR-1.Theta.MER34b</t>
-  </si>
-  <si>
-    <t>ERVR-1.Zeta.MER41</t>
-  </si>
-  <si>
-    <t>ERVR-1.Zeta.MER57</t>
-  </si>
-  <si>
-    <t>ERVR-1.Theta.MER61</t>
-  </si>
-  <si>
-    <t>ERVR-1.Unclassified.MER65</t>
-  </si>
-  <si>
     <t>ERVR-3.Lambda.70</t>
   </si>
   <si>
@@ -299,23 +182,47 @@
     <t>HERV-L74</t>
   </si>
   <si>
-    <t>ERV-3.Lambda.74</t>
-  </si>
-  <si>
     <t>ERVL47</t>
   </si>
   <si>
     <t>ERV-L47</t>
   </si>
   <si>
-    <t>ERV-3.Lambda.47</t>
+    <t>ERVR-3.Lambda.76</t>
+  </si>
+  <si>
+    <t>ERVR-1.Zeta.HF.19</t>
+  </si>
+  <si>
+    <t>ERVR-1.Zeta.W9P.P.G25</t>
+  </si>
+  <si>
+    <t>ERVR-3.Lambda.16</t>
+  </si>
+  <si>
+    <t>ERVR-3.Lambda.40</t>
+  </si>
+  <si>
+    <t>ERVR-3.Lambda.53</t>
+  </si>
+  <si>
+    <t>ERVR-3.Lambda.74</t>
+  </si>
+  <si>
+    <t>ERVR-1.Theta.24.101</t>
+  </si>
+  <si>
+    <t>ERVR-1.Theta.24.LOR1</t>
+  </si>
+  <si>
+    <t>ERVR-3.Sigma.47</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -327,6 +234,12 @@
       <b/>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -682,7 +595,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A74414C0-0D01-9B4D-8A37-18FCBAAA5CE9}">
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="35.1640625" customWidth="1"/>
@@ -694,7 +607,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>62</v>
+        <v>40</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
@@ -708,16 +621,16 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>4</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>6</v>
@@ -725,16 +638,16 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>4</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>6</v>
@@ -742,16 +655,16 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>67</v>
+        <v>42</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>4</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>6</v>
@@ -759,16 +672,16 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
-        <v>68</v>
+        <v>52</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>4</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>6</v>
@@ -776,50 +689,50 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
-        <v>68</v>
+        <v>44</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>16</v>
+        <v>31</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>4</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
-        <v>68</v>
+        <v>44</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>16</v>
+        <v>31</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>4</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
-        <v>64</v>
+        <v>45</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>8</v>
+        <v>35</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>4</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>9</v>
+        <v>36</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>6</v>
@@ -827,16 +740,16 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
-        <v>69</v>
+        <v>46</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>20</v>
+        <v>37</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>4</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>21</v>
+        <v>38</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>6</v>
@@ -844,33 +757,33 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
-        <v>70</v>
+        <v>46</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>22</v>
+        <v>37</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>4</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>23</v>
+        <v>39</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
-        <v>74</v>
+        <v>53</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>30</v>
+        <v>12</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>4</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>31</v>
+        <v>13</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>6</v>
@@ -878,16 +791,16 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
-        <v>72</v>
+        <v>53</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>26</v>
+        <v>12</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>4</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="E12" s="2" t="s">
         <v>6</v>
@@ -895,33 +808,33 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
-        <v>73</v>
+        <v>53</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>4</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>29</v>
+        <v>15</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
-        <v>71</v>
+        <v>54</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>4</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>6</v>
@@ -929,16 +842,16 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
-        <v>75</v>
+        <v>41</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>32</v>
+        <v>5</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>4</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>33</v>
+        <v>5</v>
       </c>
       <c r="E15" s="2" t="s">
         <v>6</v>
@@ -946,16 +859,16 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
-        <v>76</v>
+        <v>55</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>34</v>
+        <v>16</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>4</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
       <c r="E16" s="2" t="s">
         <v>6</v>
@@ -963,16 +876,16 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
-        <v>77</v>
+        <v>56</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>36</v>
+        <v>18</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>4</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>37</v>
+        <v>19</v>
       </c>
       <c r="E17" s="2" t="s">
         <v>6</v>
@@ -980,16 +893,16 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
-        <v>80</v>
+        <v>43</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>43</v>
+        <v>26</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>4</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>44</v>
+        <v>27</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>6</v>
@@ -997,27 +910,27 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
-        <v>81</v>
+        <v>43</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="C19" s="2" t="s">
         <v>4</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>46</v>
+        <v>28</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
-        <v>81</v>
+        <v>57</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="C20" s="2" t="s">
         <v>4</v>
@@ -1026,21 +939,21 @@
         <v>47</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A21" s="2" t="s">
-        <v>78</v>
+      <c r="A21" t="s">
+        <v>51</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>38</v>
+        <v>29</v>
       </c>
       <c r="C21" s="2" t="s">
         <v>4</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="E21" s="2" t="s">
         <v>6</v>
@@ -1048,229 +961,26 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
-        <v>79</v>
+        <v>60</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="C22" s="2" t="s">
         <v>4</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="E22" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A23" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="E23" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A24" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D24" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="E24" s="2" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A25" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="E25" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A26" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="B26" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D26" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="E26" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A27" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="B27" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D27" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="E27" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A28" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="B28" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="C28" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D28" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="E28" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A29" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="B29" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C29" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D29" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="E29" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A30" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="B30" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="C30" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D30" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="E30" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A31" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="B31" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="C31" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D31" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="E31" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A32" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="B32" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="C32" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D32" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="E32" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A33" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="B33" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="C33" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D33" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="E33" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A34" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="B34" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="C34" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D34" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="E34" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E32">
-    <sortCondition ref="A2:A32"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E22">
+    <sortCondition ref="A2:A22"/>
   </sortState>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>